<commit_message>
COLUMN: name the stiffeners after the column, not the beam
The two default rows read "beam top flange" and "beam bottom flange". The
offset IS a beam flange height - that is what it is for - but naming the plate
after the beam made it look like part of the beam, and it is not: it is welded
inside the column and it is the column's steel. They now read "upper
stiffener" and "lower stiffener". Where the height came from is still on the
sheet, in the check row's "beam flange at ±".

Adds the same 25-character guard the connection notes have, column D being 26
wide with a filled neighbour, so Excel clips rather than spills.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EnGhhpynbq7sNRTi2ok7Eu
</commit_message>
<xml_diff>
--- a/plate3d/PLATE3D_COLUMN.xlsx
+++ b/plate3d/PLATE3D_COLUMN.xlsx
@@ -131,13 +131,13 @@
     <t>1</t>
   </si>
   <si>
-    <t>beam top flange</t>
+    <t>upper stiffener</t>
   </si>
   <si>
     <t>2</t>
   </si>
   <si>
-    <t>beam bottom flange</t>
+    <t>lower stiffener</t>
   </si>
   <si>
     <t>3</t>

</xml_diff>